<commit_message>
Actualiza planificador y recetario
</commit_message>
<xml_diff>
--- a/base_platos_editable.xlsx
+++ b/base_platos_editable.xlsx
@@ -357,7 +357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:P81"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="21.14453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38.57" customWidth="1" style="2" min="1" max="1"/>
@@ -435,6 +435,16 @@
           <t>ingrediente_12</t>
         </is>
       </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>ingrediente_13</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>ingrediente_14</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="3">
       <c r="A2" s="2" t="inlineStr">
@@ -3276,44 +3286,152 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>Empanada de hojaldre de jamón y queso</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>MACU</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>2 láminas de hojaldre</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>Jamón cocido</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>Queso</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>1 huevo batido</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr"/>
+      <c r="L79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr"/>
+      <c r="N79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Bizcocho con pepitas de chocolate</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Postres</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Plátanos</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Huevo</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Harina de avena, almendra o arroz</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Chocolate 85%</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Polvo de hornear</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Pastel de carne con puré de patata</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Carnes</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Carne picada</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Cebolla</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Zanahorias</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Ajo</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Tomate frito</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Patatas</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Mantequilla</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Leche SIN LACTOSA</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>Pimienta</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>Nuez moscada</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>Queso mozzarella</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="n"/>
+      <c r="O81" s="2" t="n"/>
+      <c r="P81" s="2" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>